<commit_message>
Highlight guided elements, keep timers near conditions, and add 30 domain-specific exams
</commit_message>
<xml_diff>
--- a/content/variants/V01/Заказ на производство.xlsx
+++ b/content/variants/V01/Заказ на производство.xlsx
@@ -16,8 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="166" formatCode="0.###"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,15 +30,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A61F32"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,9 +65,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,141 +445,184 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Продукт</t>
+          <t>Авторский учебный вариант</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Швейное производство</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Производственный заказ</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Заказ покупателя</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Дата запуска</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>V01-P01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>V01-01</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>46462</v>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Продукция</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
           <t>Количество</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Дата запуска</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Стол «Берёза»</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2027-03-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="C4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Фартук поварской</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Ресурс</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Количество</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Плановый расход</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Единица</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Панель</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Крепёж</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>упак</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Опора</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>12</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Сборка</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="C7" t="inlineStr">
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Бязь</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Тесьма</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Нить</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Раскрой</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>ч</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Обработка</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="C8" t="inlineStr">
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Пошив</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>ч</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>